<commit_message>
[fix] fitToWidth/fitToHeight 완전 해제 — 시트맞추기 비활성화
fitToPage=False만으로는 부족, fitToWidth=0/fitToHeight=0도 설정해야
엑셀이 '한 페이지에 시트 맞추기'를 해제함
→ scale=65 + Break(id=84) 수동 페이지 나누기 정상 동작

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/master_template.xlsx
+++ b/templates/master_template.xlsx
@@ -2051,7 +2051,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:Z287"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
@@ -11027,8 +11027,8 @@
     <mergeCell ref="A94:B94"/>
     <mergeCell ref="I92:K92"/>
     <mergeCell ref="A9:A16"/>
+    <mergeCell ref="A86:C86"/>
     <mergeCell ref="B49:B53"/>
-    <mergeCell ref="A86:C86"/>
     <mergeCell ref="B54:B56"/>
     <mergeCell ref="E93:H93"/>
     <mergeCell ref="A88:K88"/>
@@ -11080,7 +11080,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.15" bottom="0.15" header="0" footer="0"/>
-  <pageSetup orientation="portrait" paperSize="8" scale="65" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="8" scale="65" fitToHeight="0" fitToWidth="0"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="84" min="0" max="16383" man="1"/>
   </rowBreaks>

</xml_diff>

<commit_message>
[fix] 인쇄 설정: fitToWidth=1 + fitToHeight=0 + Break(84)
"한 페이지에 모든 열 맞추기" 모드로 설정:
- fitToPage=True, fitToWidth=1 (가로 1페이지)
- fitToHeight=0 (세로 제한 없음 → 페이지 나누기 허용)
- Row 84에서 수동 페이지 나누기
→ 1p: 보장금액~총납입보험료, 2p: 갱신/리뷰

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/master_template.xlsx
+++ b/templates/master_template.xlsx
@@ -2051,7 +2051,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr autoPageBreaks="0" fitToPage="0"/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Z287"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
@@ -11027,9 +11027,9 @@
     <mergeCell ref="A94:B94"/>
     <mergeCell ref="I92:K92"/>
     <mergeCell ref="A9:A16"/>
-    <mergeCell ref="A86:C86"/>
     <mergeCell ref="B49:B53"/>
     <mergeCell ref="B54:B56"/>
+    <mergeCell ref="A86:C86"/>
     <mergeCell ref="E93:H93"/>
     <mergeCell ref="A88:K88"/>
     <mergeCell ref="B57:B58"/>
@@ -11080,7 +11080,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.15" bottom="0.15" header="0" footer="0"/>
-  <pageSetup orientation="portrait" paperSize="8" scale="65" fitToHeight="0" fitToWidth="0"/>
+  <pageSetup orientation="portrait" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="84" min="0" max="16383" man="1"/>
   </rowBreaks>

</xml_diff>

<commit_message>
[fix] 헤더 행 높이 복원 — Row 2~7 원래 15pt, Row 5/6은 30pt
이전 커밋에서 헤더를 13pt로 줄여 상품명/납입기간 텍스트 잘림 발생
→ 원래 값 복원, 보험료 행(80~82)을 15pt로 줄여 총 높이 보전
총 높이 1365pt (A3 가용 1552pt, 여유 187pt)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/master_template.xlsx
+++ b/templates/master_template.xlsx
@@ -2064,7 +2064,7 @@
     <col width="12.6640625" customWidth="1" style="5" min="12" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="95" t="inlineStr">
         <is>
           <t>님(남/여 - 세)을 위한 보장분석</t>
@@ -2091,7 +2091,7 @@
       <c r="Y1" s="4" t="n"/>
       <c r="Z1" s="4" t="n"/>
     </row>
-    <row r="2" ht="13" customHeight="1">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="97" t="n"/>
       <c r="B2" s="98" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
       <c r="Y2" s="4" t="n"/>
       <c r="Z2" s="4" t="n"/>
     </row>
-    <row r="3" ht="13" customHeight="1">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="180" t="n"/>
       <c r="B3" s="181" t="n"/>
       <c r="C3" s="102" t="inlineStr">
@@ -2163,7 +2163,7 @@
       <c r="Y3" s="4" t="n"/>
       <c r="Z3" s="4" t="n"/>
     </row>
-    <row r="4" ht="13" customHeight="1">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="180" t="n"/>
       <c r="B4" s="181" t="n"/>
       <c r="C4" s="98" t="inlineStr">
@@ -2195,7 +2195,7 @@
       <c r="Y4" s="4" t="n"/>
       <c r="Z4" s="4" t="n"/>
     </row>
-    <row r="5" ht="13" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="180" t="n"/>
       <c r="B5" s="181" t="n"/>
       <c r="C5" s="102" t="inlineStr">
@@ -2227,7 +2227,7 @@
       <c r="Y5" s="4" t="n"/>
       <c r="Z5" s="4" t="n"/>
     </row>
-    <row r="6" ht="13" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="180" t="n"/>
       <c r="B6" s="182" t="n"/>
       <c r="C6" s="98" t="inlineStr">
@@ -2259,7 +2259,7 @@
       <c r="Y6" s="4" t="n"/>
       <c r="Z6" s="4" t="n"/>
     </row>
-    <row r="7" ht="13" customHeight="1">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="180" t="n"/>
       <c r="B7" s="102" t="inlineStr">
         <is>
@@ -3074,7 +3074,7 @@
       <c r="Y29" s="4" t="n"/>
       <c r="Z29" s="4" t="n"/>
     </row>
-    <row r="30" ht="27" customHeight="1">
+    <row r="30" ht="25" customHeight="1">
       <c r="A30" s="181" t="n"/>
       <c r="B30" s="118" t="inlineStr">
         <is>
@@ -3114,7 +3114,7 @@
       <c r="Y30" s="4" t="n"/>
       <c r="Z30" s="4" t="n"/>
     </row>
-    <row r="31" ht="27" customHeight="1">
+    <row r="31" ht="25" customHeight="1">
       <c r="A31" s="181" t="n"/>
       <c r="B31" s="181" t="n"/>
       <c r="C31" s="118" t="inlineStr">
@@ -3150,7 +3150,7 @@
       <c r="Y31" s="4" t="n"/>
       <c r="Z31" s="4" t="n"/>
     </row>
-    <row r="32" ht="27" customHeight="1">
+    <row r="32" ht="25" customHeight="1">
       <c r="A32" s="181" t="n"/>
       <c r="B32" s="181" t="n"/>
       <c r="C32" s="121" t="inlineStr">
@@ -3186,7 +3186,7 @@
       <c r="Y32" s="4" t="n"/>
       <c r="Z32" s="4" t="n"/>
     </row>
-    <row r="33" ht="27" customHeight="1">
+    <row r="33" ht="25" customHeight="1">
       <c r="A33" s="181" t="n"/>
       <c r="B33" s="181" t="n"/>
       <c r="C33" s="118" t="inlineStr">
@@ -3222,7 +3222,7 @@
       <c r="Y33" s="4" t="n"/>
       <c r="Z33" s="4" t="n"/>
     </row>
-    <row r="34" ht="27" customHeight="1">
+    <row r="34" ht="25" customHeight="1">
       <c r="A34" s="182" t="n"/>
       <c r="B34" s="182" t="n"/>
       <c r="C34" s="121" t="inlineStr">
@@ -3758,7 +3758,7 @@
       <c r="Y48" s="4" t="n"/>
       <c r="Z48" s="4" t="n"/>
     </row>
-    <row r="49" ht="27" customHeight="1">
+    <row r="49" ht="25" customHeight="1">
       <c r="A49" s="222" t="n"/>
       <c r="B49" s="222" t="inlineStr">
         <is>
@@ -3781,7 +3781,7 @@
       <c r="J49" s="224" t="n"/>
       <c r="K49" s="224" t="n"/>
     </row>
-    <row r="50" ht="27" customHeight="1">
+    <row r="50" ht="25" customHeight="1">
       <c r="A50" s="227" t="n"/>
       <c r="B50" s="227" t="n"/>
       <c r="C50" s="225" t="inlineStr">
@@ -3799,7 +3799,7 @@
       <c r="J50" s="226" t="n"/>
       <c r="K50" s="226" t="n"/>
     </row>
-    <row r="51" ht="27" customHeight="1">
+    <row r="51" ht="25" customHeight="1">
       <c r="A51" s="227" t="n"/>
       <c r="B51" s="227" t="n"/>
       <c r="C51" s="223" t="inlineStr">
@@ -3817,7 +3817,7 @@
       <c r="J51" s="224" t="n"/>
       <c r="K51" s="224" t="n"/>
     </row>
-    <row r="52" ht="27" customHeight="1">
+    <row r="52" ht="25" customHeight="1">
       <c r="A52" s="227" t="n"/>
       <c r="B52" s="227" t="n"/>
       <c r="C52" s="225" t="inlineStr">
@@ -3835,7 +3835,7 @@
       <c r="J52" s="226" t="n"/>
       <c r="K52" s="226" t="n"/>
     </row>
-    <row r="53" ht="27" customHeight="1">
+    <row r="53" ht="25" customHeight="1">
       <c r="A53" s="228" t="n"/>
       <c r="B53" s="228" t="n"/>
       <c r="C53" s="223" t="inlineStr">
@@ -4791,7 +4791,7 @@
       <c r="Y79" s="4" t="n"/>
       <c r="Z79" s="4" t="n"/>
     </row>
-    <row r="80" ht="18" customHeight="1">
+    <row r="80" ht="15" customHeight="1">
       <c r="A80" s="158" t="n"/>
       <c r="B80" s="159" t="inlineStr">
         <is>
@@ -4828,7 +4828,7 @@
       <c r="Y80" s="4" t="n"/>
       <c r="Z80" s="4" t="n"/>
     </row>
-    <row r="81" ht="18" customHeight="1">
+    <row r="81" ht="15" customHeight="1">
       <c r="A81" s="181" t="n"/>
       <c r="B81" s="162" t="inlineStr">
         <is>
@@ -4865,7 +4865,7 @@
       <c r="Y81" s="4" t="n"/>
       <c r="Z81" s="4" t="n"/>
     </row>
-    <row r="82" ht="18" customHeight="1">
+    <row r="82" ht="15" customHeight="1">
       <c r="A82" s="182" t="n"/>
       <c r="B82" s="159" t="inlineStr">
         <is>
@@ -11033,8 +11033,8 @@
     <mergeCell ref="I92:K92"/>
     <mergeCell ref="A9:A16"/>
     <mergeCell ref="B49:B53"/>
+    <mergeCell ref="A86:C86"/>
     <mergeCell ref="B54:B56"/>
-    <mergeCell ref="A86:C86"/>
     <mergeCell ref="E93:H93"/>
     <mergeCell ref="A88:K88"/>
     <mergeCell ref="B57:B58"/>
@@ -11084,7 +11084,7 @@
     <mergeCell ref="K2:K6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.15" header="0" footer="0"/>
+  <pageMargins left="0.3" right="0.3" top="0.2" bottom="0.15" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="84" min="0" max="16383" man="1"/>

</xml_diff>